<commit_message>
High vs Storm Water Level graphs
</commit_message>
<xml_diff>
--- a/oahu_windward_beaches_microplastics_survey.xlsx
+++ b/oahu_windward_beaches_microplastics_survey.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10913"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jd/Desktop/Data Science Masters Coursework/Fall 2026/STA 6349/Project/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/joshuadilena/Library/Mobile Documents/com~apple~CloudDocs/Desktop/Data Science Masters Coursework/Fall 2026/STA 6349/STA6349-Project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC208685-C464-3C45-BACD-DE4AD45395F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ECAB5FE-E33F-6544-914F-6AD950427AA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="16940" xr2:uid="{B0BDD1F7-4A5A-3B45-B26A-32EF93B12A14}"/>
+    <workbookView xWindow="16560" yWindow="3880" windowWidth="28040" windowHeight="16940" xr2:uid="{B0BDD1F7-4A5A-3B45-B26A-32EF93B12A14}"/>
   </bookViews>
   <sheets>
     <sheet name="Particles per Quad" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Medians added to scatter plot
</commit_message>
<xml_diff>
--- a/oahu_windward_beaches_microplastics_survey.xlsx
+++ b/oahu_windward_beaches_microplastics_survey.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10913"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/joshuadilena/Library/Mobile Documents/com~apple~CloudDocs/Desktop/Data Science Masters Coursework/Fall 2026/STA 6349/STA6349-Project/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jdilena\Documents\Github Repos\STA6349-Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ECAB5FE-E33F-6544-914F-6AD950427AA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBEC8A91-76DE-4AF0-ABFE-91EAF15AFD03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16560" yWindow="3880" windowWidth="28040" windowHeight="16940" xr2:uid="{B0BDD1F7-4A5A-3B45-B26A-32EF93B12A14}"/>
+    <workbookView xWindow="-27630" yWindow="-135" windowWidth="21600" windowHeight="11295" xr2:uid="{B0BDD1F7-4A5A-3B45-B26A-32EF93B12A14}"/>
   </bookViews>
   <sheets>
     <sheet name="Particles per Quad" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,20 @@
     <sheet name="Beach Location" sheetId="4" r:id="rId3"/>
     <sheet name="Percent Particles per Size Clas" sheetId="2" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -974,12 +987,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BAF9EA0-6F22-3C4B-84BA-D9626617907D}">
   <dimension ref="A1:C109"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="30.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="30.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -990,7 +1003,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -1001,7 +1014,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -1012,7 +1025,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>2</v>
       </c>
@@ -1023,7 +1036,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -1034,7 +1047,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -1045,7 +1058,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>2</v>
       </c>
@@ -1056,7 +1069,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>2</v>
       </c>
@@ -1067,7 +1080,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>2</v>
       </c>
@@ -1078,7 +1091,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>2</v>
       </c>
@@ -1089,7 +1102,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>2</v>
       </c>
@@ -1100,7 +1113,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>2</v>
       </c>
@@ -1111,7 +1124,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>2</v>
       </c>
@@ -1122,7 +1135,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>2</v>
       </c>
@@ -1133,7 +1146,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>2</v>
       </c>
@@ -1144,7 +1157,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>2</v>
       </c>
@@ -1155,7 +1168,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>2</v>
       </c>
@@ -1166,7 +1179,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>2</v>
       </c>
@@ -1177,7 +1190,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>2</v>
       </c>
@@ -1188,7 +1201,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>5</v>
       </c>
@@ -1199,7 +1212,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>5</v>
       </c>
@@ -1210,7 +1223,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>5</v>
       </c>
@@ -1221,7 +1234,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>5</v>
       </c>
@@ -1232,7 +1245,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>5</v>
       </c>
@@ -1243,7 +1256,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>5</v>
       </c>
@@ -1254,7 +1267,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>5</v>
       </c>
@@ -1265,7 +1278,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>5</v>
       </c>
@@ -1276,7 +1289,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>5</v>
       </c>
@@ -1287,7 +1300,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>5</v>
       </c>
@@ -1298,7 +1311,7 @@
         <v>1067</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>5</v>
       </c>
@@ -1309,7 +1322,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>5</v>
       </c>
@@ -1320,7 +1333,7 @@
         <v>1956</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>5</v>
       </c>
@@ -1331,7 +1344,7 @@
         <v>722</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>5</v>
       </c>
@@ -1342,7 +1355,7 @@
         <v>1678</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>5</v>
       </c>
@@ -1353,7 +1366,7 @@
         <v>1756</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>5</v>
       </c>
@@ -1364,7 +1377,7 @@
         <v>1567</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>5</v>
       </c>
@@ -1375,7 +1388,7 @@
         <v>811</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>5</v>
       </c>
@@ -1386,7 +1399,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>6</v>
       </c>
@@ -1397,7 +1410,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>6</v>
       </c>
@@ -1408,7 +1421,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>6</v>
       </c>
@@ -1419,7 +1432,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>6</v>
       </c>
@@ -1430,7 +1443,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>6</v>
       </c>
@@ -1441,7 +1454,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>6</v>
       </c>
@@ -1452,7 +1465,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>6</v>
       </c>
@@ -1463,7 +1476,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>6</v>
       </c>
@@ -1474,7 +1487,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>6</v>
       </c>
@@ -1485,7 +1498,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>6</v>
       </c>
@@ -1496,7 +1509,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>6</v>
       </c>
@@ -1507,7 +1520,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>6</v>
       </c>
@@ -1518,7 +1531,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>6</v>
       </c>
@@ -1529,7 +1542,7 @@
         <v>1922</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>6</v>
       </c>
@@ -1540,7 +1553,7 @@
         <v>833</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>6</v>
       </c>
@@ -1551,7 +1564,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>6</v>
       </c>
@@ -1562,7 +1575,7 @@
         <v>1200</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>6</v>
       </c>
@@ -1573,7 +1586,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>6</v>
       </c>
@@ -1584,7 +1597,7 @@
         <v>1122</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>7</v>
       </c>
@@ -1595,7 +1608,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>7</v>
       </c>
@@ -1606,7 +1619,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>7</v>
       </c>
@@ -1617,7 +1630,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>7</v>
       </c>
@@ -1628,7 +1641,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>7</v>
       </c>
@@ -1639,7 +1652,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>7</v>
       </c>
@@ -1650,7 +1663,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>7</v>
       </c>
@@ -1661,7 +1674,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>7</v>
       </c>
@@ -1672,7 +1685,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>7</v>
       </c>
@@ -1683,7 +1696,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>7</v>
       </c>
@@ -1694,7 +1707,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>7</v>
       </c>
@@ -1705,7 +1718,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>7</v>
       </c>
@@ -1716,7 +1729,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>7</v>
       </c>
@@ -1727,7 +1740,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>7</v>
       </c>
@@ -1738,7 +1751,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>7</v>
       </c>
@@ -1749,7 +1762,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>7</v>
       </c>
@@ -1760,7 +1773,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>7</v>
       </c>
@@ -1771,7 +1784,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>7</v>
       </c>
@@ -1782,7 +1795,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>8</v>
       </c>
@@ -1793,7 +1806,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>8</v>
       </c>
@@ -1804,7 +1817,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>8</v>
       </c>
@@ -1815,7 +1828,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>8</v>
       </c>
@@ -1826,7 +1839,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>8</v>
       </c>
@@ -1837,7 +1850,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>8</v>
       </c>
@@ -1848,7 +1861,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>8</v>
       </c>
@@ -1859,7 +1872,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>8</v>
       </c>
@@ -1870,7 +1883,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>8</v>
       </c>
@@ -1881,7 +1894,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>8</v>
       </c>
@@ -1892,7 +1905,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>8</v>
       </c>
@@ -1903,7 +1916,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>8</v>
       </c>
@@ -1914,7 +1927,7 @@
         <v>789</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>8</v>
       </c>
@@ -1925,7 +1938,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>8</v>
       </c>
@@ -1936,7 +1949,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>8</v>
       </c>
@@ -1947,7 +1960,7 @@
         <v>278</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>8</v>
       </c>
@@ -1958,7 +1971,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>8</v>
       </c>
@@ -1969,7 +1982,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>8</v>
       </c>
@@ -1980,7 +1993,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>9</v>
       </c>
@@ -1991,7 +2004,7 @@
         <v>1333</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>9</v>
       </c>
@@ -2002,7 +2015,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>9</v>
       </c>
@@ -2013,7 +2026,7 @@
         <v>844</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>9</v>
       </c>
@@ -2024,7 +2037,7 @@
         <v>3467</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>9</v>
       </c>
@@ -2035,7 +2048,7 @@
         <v>1689</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>9</v>
       </c>
@@ -2046,7 +2059,7 @@
         <v>2800</v>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>9</v>
       </c>
@@ -2057,7 +2070,7 @@
         <v>2800</v>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>9</v>
       </c>
@@ -2068,7 +2081,7 @@
         <v>1778</v>
       </c>
     </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>9</v>
       </c>
@@ -2079,7 +2092,7 @@
         <v>1289</v>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>9</v>
       </c>
@@ -2090,7 +2103,7 @@
         <v>3289</v>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>9</v>
       </c>
@@ -2101,7 +2114,7 @@
         <v>2533</v>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>9</v>
       </c>
@@ -2112,7 +2125,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>9</v>
       </c>
@@ -2123,7 +2136,7 @@
         <v>844</v>
       </c>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>9</v>
       </c>
@@ -2134,7 +2147,7 @@
         <v>1111</v>
       </c>
     </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>9</v>
       </c>
@@ -2145,7 +2158,7 @@
         <v>1422</v>
       </c>
     </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>9</v>
       </c>
@@ -2156,7 +2169,7 @@
         <v>1911</v>
       </c>
     </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>9</v>
       </c>
@@ -2167,7 +2180,7 @@
         <v>1467</v>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>9</v>
       </c>
@@ -2186,13 +2199,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DB8A044-DF37-6240-861D-B6DB238C7141}">
   <dimension ref="A1:H7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.875" customWidth="1"/>
+    <col min="4" max="4" width="12.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2218,7 +2231,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -2244,7 +2257,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -2270,7 +2283,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -2296,7 +2309,7 @@
         <v>0.06</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -2322,7 +2335,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -2348,7 +2361,7 @@
         <v>0.03</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2382,9 +2395,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AD79E026-E7A1-E54E-AAC5-BD3B6A1B6CF8}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>21</v>
       </c>
@@ -2395,7 +2408,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -2406,7 +2419,7 @@
         <v>21.68</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>25</v>
       </c>
@@ -2417,7 +2430,7 @@
         <v>21.4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>26</v>
       </c>
@@ -2428,7 +2441,7 @@
         <v>21.39</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -2439,7 +2452,7 @@
         <v>21.34</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>28</v>
       </c>
@@ -2450,7 +2463,7 @@
         <v>21.326000000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>29</v>
       </c>
@@ -2469,9 +2482,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9888261E-4C14-6A44-B6E8-8786D8CB19BE}">
   <dimension ref="A1:E13"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2488,7 +2501,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -2505,7 +2518,7 @@
         <v>27.3</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -2522,7 +2535,7 @@
         <v>20.5</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -2539,7 +2552,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -2556,7 +2569,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -2573,7 +2586,7 @@
         <v>8.1</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2590,7 +2603,7 @@
         <v>5.2</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>2</v>
       </c>
@@ -2607,7 +2620,7 @@
         <v>14.9</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -2624,7 +2637,7 @@
         <v>10.9</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>6</v>
       </c>
@@ -2641,7 +2654,7 @@
         <v>11.6</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>7</v>
       </c>
@@ -2658,7 +2671,7 @@
         <v>6.4</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>8</v>
       </c>
@@ -2675,7 +2688,7 @@
         <v>6.3</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>9</v>
       </c>

</xml_diff>